<commit_message>
Móvil con sección y marcador; arreglo al saltar de sección; sin Spotify
- Móvil del concursante: barra con la sección en curso (nº, tipo,
  pregunta/ronda/prueba, puntos en juego y descripción) y su equipo con
  el puesto. Tocando sus puntos se abre el marcador en directo (equipos
  y concursantes, con los suyos resaltados) sin salir del juego.
- Tele: al saltar de sección ya no se queda encima el ganador del
  pulsador, ni relojes ni la luz de Reflejos de la pantalla anterior.
- Spotify descartado: fuera del plan y de la plantilla (columnas de
  música y canción); las hojas antiguas que las traigan se aceptan.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantilla-concurso.xlsx
+++ b/public/plantilla-concurso.xlsx
@@ -138,13 +138,6 @@
         </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="0">
-      <text>
-        <r>
-          <t>Opcional: enlace a una canción de Spotify.</t>
-        </r>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
@@ -194,13 +187,6 @@
       </text>
     </comment>
     <comment ref="E1" authorId="0">
-      <text>
-        <r>
-          <t>Opcional: enlace de Spotify. Se pausa sola cuando alguien pulsa.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0">
       <text>
         <r>
           <t>Solo para ti.</t>
@@ -284,7 +270,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="134">
   <si>
     <t>CÓMO RELLENAR ESTA PLANTILLA</t>
   </si>
@@ -316,9 +302,6 @@
     <t>6. Puntos: un número (por acierto) o una lista por puestos, como 3,2,1 (1º, 2º y 3º).</t>
   </si>
   <si>
-    <t>7. Canciones: copia el enlace de Spotify (Compartir → Copiar enlace de la canción).</t>
-  </si>
-  <si>
     <t>Para cargarla: en el portátil, pantalla de preparación → "Cargar concurso" → elige este archivo.</t>
   </si>
   <si>
@@ -346,9 +329,6 @@
     <t>El presentador juega</t>
   </si>
   <si>
-    <t>Música de entrada</t>
-  </si>
-  <si>
     <t>Calentamiento</t>
   </si>
   <si>
@@ -436,9 +416,6 @@
     <t>Sí</t>
   </si>
   <si>
-    <t>https://open.spotify.com/track/4uLU6hMCjMI75M1A2tKUQC</t>
-  </si>
-  <si>
     <t>Equipo</t>
   </si>
   <si>
@@ -499,12 +476,6 @@
     <t>Mostrar en tele</t>
   </si>
   <si>
-    <t>Canción</t>
-  </si>
-  <si>
-    <t>Desde segundo</t>
-  </si>
-  <si>
     <t>Notas</t>
   </si>
   <si>
@@ -520,13 +491,13 @@
     <t>Ocho</t>
   </si>
   <si>
-    <t>¿Qué canción es?</t>
-  </si>
-  <si>
-    <t>Mr. Brightside</t>
-  </si>
-  <si>
-    <t>Suena 20 s</t>
+    <t>🎵 ¿Qué canción suena?</t>
+  </si>
+  <si>
+    <t>Mr. Brightside (The Killers)</t>
+  </si>
+  <si>
+    <t>Pon la canción tú desde tu música</t>
   </si>
   <si>
     <t>A</t>
@@ -1101,7 +1072,7 @@
   <sheetPr>
     <tabColor rgb="FF111111"/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -1159,12 +1130,12 @@
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
@@ -1175,11 +1146,6 @@
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>12</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -1205,53 +1171,53 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="C2">
         <v>910</v>
       </c>
       <c r="D2" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="E2" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B3" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="C3">
         <v>120</v>
       </c>
       <c r="D3" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="E3" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25"/>
@@ -1487,38 +1453,38 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B2">
         <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B3">
         <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="D3">
         <v>3</v>
@@ -1526,13 +1492,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B4">
         <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25"/>
@@ -1767,24 +1733,24 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B2">
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25"/>
@@ -2023,56 +1989,56 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>17</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B2" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="C2" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="D2" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="E2" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B3" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="C3" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="D3" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="E3" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="F3">
         <v>5</v>
@@ -2307,7 +2273,7 @@
   <sheetPr>
     <tabColor rgb="FFFFD400"/>
   </sheetPr>
-  <dimension ref="A1:G200"/>
+  <dimension ref="A1:F200"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -2315,192 +2281,185 @@
     <col min="4" max="4" width="50" customWidth="1"/>
     <col min="5" max="5" width="10" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
-    <col min="7" max="7" width="46" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" t="s">
         <v>21</v>
-      </c>
-      <c r="C2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D2" t="s">
-        <v>23</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" t="s">
         <v>25</v>
-      </c>
-      <c r="C3" t="s">
-        <v>26</v>
-      </c>
-      <c r="D3" t="s">
-        <v>27</v>
       </c>
       <c r="E3">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" t="s">
         <v>28</v>
-      </c>
-      <c r="C4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D4" t="s">
-        <v>30</v>
       </c>
       <c r="E4">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" t="s">
         <v>31</v>
-      </c>
-      <c r="C5" t="s">
-        <v>32</v>
-      </c>
-      <c r="D5" t="s">
-        <v>33</v>
       </c>
       <c r="E5">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" t="s">
         <v>34</v>
       </c>
-      <c r="C6" t="s">
+      <c r="E6" t="s">
         <v>35</v>
       </c>
-      <c r="D6" t="s">
-        <v>36</v>
-      </c>
-      <c r="E6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" t="s">
         <v>38</v>
       </c>
-      <c r="C7" t="s">
-        <v>39</v>
-      </c>
-      <c r="D7" t="s">
-        <v>40</v>
-      </c>
       <c r="E7" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" t="s">
         <v>41</v>
       </c>
-      <c r="C8" t="s">
-        <v>42</v>
-      </c>
-      <c r="D8" t="s">
-        <v>43</v>
-      </c>
       <c r="E8" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C9" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D9" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E9">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" t="s">
         <v>46</v>
-      </c>
-      <c r="C10" t="s">
-        <v>47</v>
-      </c>
-      <c r="D10" t="s">
-        <v>48</v>
       </c>
       <c r="E10">
         <v>3</v>
       </c>
       <c r="F10" t="s">
-        <v>49</v>
-      </c>
-      <c r="G10" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" spans="3:6" x14ac:dyDescent="0.25"/>
@@ -2728,26 +2687,26 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B3" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.25"/>
@@ -2976,23 +2935,23 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -3000,7 +2959,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -3008,7 +2967,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -3016,7 +2975,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -3024,7 +2983,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -3032,15 +2991,15 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B8" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B9">
         <v>20</v>
@@ -3057,90 +3016,76 @@
   <sheetPr>
     <tabColor rgb="FFE53935"/>
   </sheetPr>
-  <dimension ref="A1:G200"/>
+  <dimension ref="A1:E200"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
     <col min="3" max="3" width="30" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="5" max="5" width="46" customWidth="1"/>
-    <col min="6" max="6" width="10" customWidth="1"/>
-    <col min="7" max="7" width="30" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="3" t="s">
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" t="s">
         <v>69</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="C2" t="s">
         <v>70</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="D2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" t="s">
         <v>71</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="C3" t="s">
         <v>72</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="D3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="C4" t="s">
         <v>74</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E4" t="s">
         <v>75</v>
-      </c>
-      <c r="D2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C3" t="s">
-        <v>77</v>
-      </c>
-      <c r="D3" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" t="s">
-        <v>78</v>
-      </c>
-      <c r="C4" t="s">
-        <v>79</v>
-      </c>
-      <c r="D4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E4" t="s">
-        <v>50</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25"/>
@@ -3377,74 +3322,74 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>82</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="C2" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D2" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="E2" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="F2" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="G2" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="C3" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="D3" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="E3" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="G3" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="H3">
         <v>15</v>
@@ -3683,35 +3628,35 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B2" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="C2" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="C3" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25"/>
@@ -3947,39 +3892,39 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B2" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="C2" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="D2" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="E2" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="F2">
         <v>2</v>
@@ -4218,26 +4163,26 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B2" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B3" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Fase 9: espectáculo con tema de Halloween
- Entorno animado por sección en la tele (WebGL): cementerio, bosque, calabazas,
  laboratorio, mansión, telaraña, aquelarre, cripta, tormenta y noche de luna.
  Columna opcional «Entorno» en la hoja; los móviles usan sus colores de fondo.
- Música ambiental y efectos generados con Web Audio (sin archivos), con
  ajustes de música, efectos y volumen en la tele y en el mando.
- Transiciones, títulos letra a letra, puntos que ruedan, marcador que se
  reordena, revelados con suspense, podio con confeti.
- Tarjetas compactas para muchos jugadores, wake lock en los móviles.
- h() aplica las variables CSS de style (antes se perdían los colores).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantilla-concurso.xlsx
+++ b/public/plantilla-concurso.xlsx
@@ -138,6 +138,13 @@
         </r>
       </text>
     </comment>
+    <comment ref="G1" authorId="0">
+      <text>
+        <r>
+          <t>Decorado de Halloween de la tele en esta sección. Vacío = uno distinto en cada sección.</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -270,7 +277,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="136">
   <si>
     <t>CÓMO RELLENAR ESTA PLANTILLA</t>
   </si>
@@ -329,6 +336,9 @@
     <t>El presentador juega</t>
   </si>
   <si>
+    <t>Entorno</t>
+  </si>
+  <si>
     <t>Calentamiento</t>
   </si>
   <si>
@@ -414,6 +424,9 @@
   </si>
   <si>
     <t>Sí</t>
+  </si>
+  <si>
+    <t>Noche de luna</t>
   </si>
   <si>
     <t>Equipo</t>
@@ -1174,50 +1187,50 @@
         <v>14</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C2">
         <v>910</v>
       </c>
       <c r="D2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B3" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C3">
         <v>120</v>
       </c>
       <c r="D3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E3" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25"/>
@@ -1456,35 +1469,35 @@
         <v>14</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B2">
         <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B3">
         <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D3">
         <v>3</v>
@@ -1492,13 +1505,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B4">
         <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25"/>
@@ -1736,21 +1749,21 @@
         <v>14</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B2">
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25"/>
@@ -1992,16 +2005,16 @@
         <v>14</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>17</v>
@@ -2009,36 +2022,36 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C2" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D2" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E3" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="F3">
         <v>5</v>
@@ -2273,7 +2286,7 @@
   <sheetPr>
     <tabColor rgb="FFFFD400"/>
   </sheetPr>
-  <dimension ref="A1:F200"/>
+  <dimension ref="A1:G200"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -2281,9 +2294,10 @@
     <col min="4" max="4" width="50" customWidth="1"/>
     <col min="5" max="5" width="10" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>13</v>
       </c>
@@ -2302,358 +2316,364 @@
       <c r="F1" s="3" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E3">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E4">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E5">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E6" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7" t="s">
         <v>36</v>
       </c>
-      <c r="C7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D7" t="s">
-        <v>38</v>
-      </c>
-      <c r="E7" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E8" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E9">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C10" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E10">
         <v>3</v>
       </c>
       <c r="F10" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="11" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="17" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="18" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="19" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="20" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="33" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="34" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="35" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="36" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="37" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="40" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="49" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="50" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="51" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="52" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="53" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="54" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="55" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="57" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="60" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="61" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="62" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="63" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="65" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="66" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="67" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="68" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="69" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="70" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="71" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="72" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="73" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="74" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="75" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="76" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="77" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="78" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="79" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="80" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="81" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="82" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="83" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="84" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="85" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="86" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="87" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="88" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="89" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="90" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="91" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="92" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="93" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="94" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="95" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="96" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="97" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="98" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="99" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="100" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="101" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="102" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="103" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="104" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="105" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="106" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="107" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="108" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="109" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="110" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="111" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="112" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="113" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="114" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="115" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="116" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="117" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="118" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="119" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="120" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="121" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="122" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="123" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="124" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="125" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="126" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="127" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="128" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="129" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="130" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="131" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="132" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="133" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="134" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="135" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="136" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="137" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="138" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="139" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="140" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="141" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="142" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="143" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="144" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="145" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="146" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="147" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="148" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="149" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="150" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="151" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="152" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="153" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="154" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="155" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="156" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="157" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="158" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="159" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="160" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="161" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="162" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="163" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="164" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="165" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="166" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="167" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="168" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="169" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="170" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="171" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="172" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="173" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="174" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="175" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="176" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="177" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="178" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="179" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="180" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="181" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="182" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="183" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="184" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="185" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="186" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="187" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="188" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="189" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="190" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="191" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="192" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="193" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="194" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="195" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="196" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="197" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="198" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="199" spans="3:6" x14ac:dyDescent="0.25"/>
-    <row r="200" spans="3:6" x14ac:dyDescent="0.25"/>
+        <v>48</v>
+      </c>
+      <c r="G10" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="11" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="17" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="18" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="19" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="20" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="21" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="22" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="33" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="34" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="35" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="36" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="37" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="40" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="43" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="45" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="46" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="48" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="49" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="50" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="51" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="52" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="53" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="54" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="55" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="56" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="57" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="58" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="59" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="60" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="61" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="62" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="63" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="64" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="65" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="66" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="67" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="68" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="69" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="70" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="71" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="72" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="73" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="74" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="75" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="76" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="77" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="78" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="79" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="80" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="81" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="82" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="83" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="84" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="85" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="86" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="87" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="88" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="89" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="90" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="91" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="92" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="93" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="94" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="95" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="96" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="97" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="98" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="99" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="100" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="101" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="102" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="103" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="104" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="105" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="106" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="107" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="108" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="109" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="110" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="111" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="112" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="113" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="114" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="115" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="116" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="117" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="118" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="119" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="120" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="121" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="122" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="123" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="124" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="125" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="126" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="127" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="128" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="129" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="130" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="131" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="132" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="133" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="134" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="135" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="136" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="137" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="138" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="139" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="140" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="141" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="142" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="143" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="144" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="145" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="146" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="147" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="148" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="149" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="150" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="151" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="152" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="153" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="154" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="155" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="156" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="157" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="158" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="159" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="160" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="161" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="162" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="163" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="164" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="165" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="166" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="167" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="168" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="169" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="170" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="171" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="172" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="173" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="174" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="175" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="176" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="177" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="178" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="179" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="180" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="181" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="182" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="183" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="184" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="185" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="186" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="187" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="188" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="189" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="190" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="191" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="192" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="193" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="194" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="195" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="196" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="197" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="198" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="199" spans="3:7" x14ac:dyDescent="0.25"/>
+    <row r="200" spans="3:7" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <dataValidations count="4">
+  <dataValidations count="6">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="C10:C200">
       <formula1>"Pulsador,Test,Verdad o mentira,Dos verdades y una mentira,Votación,Estimación,Parar el contador,Duelo de reflejos,Libre"</formula1>
     </dataValidation>
@@ -2665,6 +2685,12 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="F2:F200">
       <formula1>"Sí,No"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="G10:G200">
+      <formula1>"Noche de luna,Cementerio,Bosque encantado,Huerto de calabazas,Laboratorio,Mansión encantada,Telaraña,Aquelarre,Cripta helada,Tormenta"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="G2:G200">
+      <formula1>"Noche de luna,Cementerio,Bosque encantado,Huerto de calabazas,Laboratorio,Mansión encantada,Telaraña,Aquelarre,Cripta helada,Tormenta"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2687,26 +2713,26 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.25"/>
@@ -2935,23 +2961,23 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -2959,7 +2985,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -2967,7 +2993,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -2975,7 +3001,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -2983,7 +3009,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -2991,15 +3017,15 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B9">
         <v>20</v>
@@ -3031,61 +3057,61 @@
         <v>14</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25"/>
@@ -3325,71 +3351,71 @@
         <v>14</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="G2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H3">
         <v>15</v>
@@ -3631,32 +3657,32 @@
         <v>14</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25"/>
@@ -3895,36 +3921,36 @@
         <v>14</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>98</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F2">
         <v>2</v>
@@ -4166,23 +4192,23 @@
         <v>14</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Millonario, antitrampas, turnos, caras y canciones por sección
- Test como «¿Quién quiere ser millonario?»: un concursante cada vez alternando
  equipos, el presentador enseña, marca (amarilla) y revela (verde); comodines
  50:50, Público (vota su equipo 15 s, anulable) y Llamada (30 s con reloj).
- Antitrampas: salir de la app con la pregunta abierta anula la respuesta.
- Por turnos con portavoz que ordena a su equipo.
- Caras de los jugadores por nombre; elegir icono y color; cambiar de sala.
- Música: huecos con nombre por sección, escalera por pregunta y efectos.
- Revelado con transición y puntos tras el suspense; despistes en Reflejos;
  un contador por equipo en Libre.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantilla-concurso.xlsx
+++ b/public/plantilla-concurso.xlsx
@@ -141,6 +141,13 @@
     <comment ref="G1" authorId="0">
       <text>
         <r>
+          <t>Sí: cada pregunta la responde un solo jugador de cada equipo. Al empezar la sección, el portavoz de cada equipo elige el orden en su móvil (de la pregunta más fácil a la más difícil). Solo Verdad o mentira, Estimación y Parar el contador, y con equipos. El Test (millonario) siempre va por turnos: un concursante cada vez, alternando equipos.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0">
+      <text>
+        <r>
           <t>Decorado de Halloween de la tele en esta sección. Vacío = uno distinto en cada sección.</t>
         </r>
       </text>
@@ -220,13 +227,6 @@
     <comment ref="H1" authorId="0">
       <text>
         <r>
-          <t>Vacío = el de Ajustes.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0">
-      <text>
-        <r>
           <t>Opcional: dirección web de una imagen.</t>
         </r>
       </text>
@@ -277,7 +277,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="147">
   <si>
     <t>CÓMO RELLENAR ESTA PLANTILLA</t>
   </si>
@@ -291,7 +291,10 @@
     <t>2. Equipos: uno por fila con su color. Si la dejas vacía, se juega sin equipos.</t>
   </si>
   <si>
-    <t>3. Ajustes: título, comodines por equipo (o por jugador si no hay equipos) y puntos por defecto.</t>
+    <t>3. Ajustes: título, comodines del Test (50:50, Público y Llamada) por equipo (o por jugador sin equipos) y puntos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   El Test se juega como «¿Quién quiere ser millonario?»: un concursante cada vez; ordena sus preguntas de fácil a difícil.</t>
   </si>
   <si>
     <t>4. Cada tipo de sección tiene su pestaña. En la columna "Sección" escribe (o elige) el nombre de la sección</t>
@@ -336,6 +339,9 @@
     <t>El presentador juega</t>
   </si>
   <si>
+    <t>Por turnos</t>
+  </si>
+  <si>
     <t>Entorno</t>
   </si>
   <si>
@@ -357,7 +363,7 @@
     <t>Test</t>
   </si>
   <si>
-    <t>Cuatro respuestas, solo una buena.</t>
+    <t>¿Quién quiere ser millonario? Uno cada vez; vuestro portavoz decide el orden.</t>
   </si>
   <si>
     <t>¿Verdad o mentira?</t>
@@ -462,7 +468,7 @@
     <t>Comodín 50 %</t>
   </si>
   <si>
-    <t>Comodín Doble</t>
+    <t>Comodín Llamada</t>
   </si>
   <si>
     <t>Comodín Público</t>
@@ -528,12 +534,21 @@
     <t>Correcta</t>
   </si>
   <si>
-    <t>Segundos</t>
-  </si>
-  <si>
     <t>Imagen</t>
   </si>
   <si>
+    <t>¿Cuántos lados tiene un hexágono?</t>
+  </si>
+  <si>
+    <t>Cinco</t>
+  </si>
+  <si>
+    <t>Seis</t>
+  </si>
+  <si>
+    <t>Siete</t>
+  </si>
+  <si>
     <t>¿En qué año llegó el hombre a la Luna?</t>
   </si>
   <si>
@@ -549,6 +564,21 @@
     <t>1975</t>
   </si>
   <si>
+    <t>¿Cuál es la capital de provincia española que está a más altura?</t>
+  </si>
+  <si>
+    <t>Cuenca</t>
+  </si>
+  <si>
+    <t>Badajoz</t>
+  </si>
+  <si>
+    <t>Jaén</t>
+  </si>
+  <si>
+    <t>Ávila</t>
+  </si>
+  <si>
     <t>¿Cuál es el planeta más grande?</t>
   </si>
   <si>
@@ -559,6 +589,9 @@
   </si>
   <si>
     <t>Júpiter</t>
+  </si>
+  <si>
+    <t>Urano</t>
   </si>
   <si>
     <t>Afirmación</t>
@@ -1085,7 +1118,7 @@
   <sheetPr>
     <tabColor rgb="FF111111"/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -1143,12 +1176,12 @@
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
@@ -1159,6 +1192,11 @@
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -1184,53 +1222,53 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>110</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B2" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
       <c r="C2">
         <v>910</v>
       </c>
       <c r="D2" t="s">
-        <v>112</v>
+        <v>123</v>
       </c>
       <c r="E2" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>114</v>
+        <v>125</v>
       </c>
       <c r="C3">
         <v>120</v>
       </c>
       <c r="D3" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="E3" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25"/>
@@ -1466,38 +1504,38 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B2">
         <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B3">
         <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="D3">
         <v>3</v>
@@ -1505,13 +1543,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B4">
         <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25"/>
@@ -1746,24 +1784,24 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B2">
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25"/>
@@ -2002,56 +2040,56 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="C2" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="D2" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="E2" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B3" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="C3" t="s">
-        <v>133</v>
+        <v>144</v>
       </c>
       <c r="D3" t="s">
-        <v>134</v>
+        <v>145</v>
       </c>
       <c r="E3" t="s">
-        <v>135</v>
+        <v>146</v>
       </c>
       <c r="F3">
         <v>5</v>
@@ -2286,7 +2324,7 @@
   <sheetPr>
     <tabColor rgb="FFFFD400"/>
   </sheetPr>
-  <dimension ref="A1:G200"/>
+  <dimension ref="A1:H200"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -2294,384 +2332,388 @@
     <col min="4" max="4" width="50" customWidth="1"/>
     <col min="5" max="5" width="10" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
-    <col min="7" max="7" width="22" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E3">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E4">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E5">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" t="s">
+        <v>41</v>
+      </c>
+      <c r="E7" t="s">
         <v>38</v>
       </c>
-      <c r="D7" t="s">
-        <v>39</v>
-      </c>
-      <c r="E7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E8" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C9" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E9">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C10" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E10">
         <v>3</v>
       </c>
       <c r="F10" t="s">
-        <v>48</v>
-      </c>
-      <c r="G10" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="11" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="17" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="18" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="19" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="20" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="33" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="34" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="35" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="36" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="37" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="40" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="49" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="50" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="51" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="52" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="53" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="54" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="55" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="57" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="60" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="61" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="62" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="63" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="65" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="66" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="67" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="68" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="69" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="70" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="71" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="72" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="73" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="74" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="75" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="76" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="77" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="78" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="79" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="80" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="81" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="82" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="83" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="84" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="85" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="86" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="87" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="88" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="89" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="90" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="91" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="92" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="93" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="94" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="95" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="96" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="97" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="98" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="99" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="100" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="101" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="102" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="103" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="104" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="105" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="106" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="107" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="108" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="109" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="110" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="111" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="112" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="113" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="114" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="115" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="116" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="117" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="118" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="119" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="120" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="121" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="122" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="123" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="124" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="125" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="126" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="127" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="128" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="129" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="130" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="131" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="132" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="133" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="134" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="135" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="136" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="137" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="138" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="139" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="140" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="141" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="142" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="143" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="144" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="145" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="146" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="147" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="148" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="149" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="150" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="151" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="152" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="153" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="154" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="155" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="156" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="157" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="158" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="159" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="160" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="161" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="162" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="163" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="164" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="165" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="166" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="167" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="168" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="169" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="170" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="171" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="172" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="173" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="174" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="175" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="176" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="177" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="178" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="179" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="180" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="181" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="182" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="183" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="184" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="185" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="186" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="187" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="188" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="189" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="190" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="191" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="192" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="193" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="194" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="195" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="196" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="197" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="198" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="199" spans="3:7" x14ac:dyDescent="0.25"/>
-    <row r="200" spans="3:7" x14ac:dyDescent="0.25"/>
+        <v>50</v>
+      </c>
+      <c r="H10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="11" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="17" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="18" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="19" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="20" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="21" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="22" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="33" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="34" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="35" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="36" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="37" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="40" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="43" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="45" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="46" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="48" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="49" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="50" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="51" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="52" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="53" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="54" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="55" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="56" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="57" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="58" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="59" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="60" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="61" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="62" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="63" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="64" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="65" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="66" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="67" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="68" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="69" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="70" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="71" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="72" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="73" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="74" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="75" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="76" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="77" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="78" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="79" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="80" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="81" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="82" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="83" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="84" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="85" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="86" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="87" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="88" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="89" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="90" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="91" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="92" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="93" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="94" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="95" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="96" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="97" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="98" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="99" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="100" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="101" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="102" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="103" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="104" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="105" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="106" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="107" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="108" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="109" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="110" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="111" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="112" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="113" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="114" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="115" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="116" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="117" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="118" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="119" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="120" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="121" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="122" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="123" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="124" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="125" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="126" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="127" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="128" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="129" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="130" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="131" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="132" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="133" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="134" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="135" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="136" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="137" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="138" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="139" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="140" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="141" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="142" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="143" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="144" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="145" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="146" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="147" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="148" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="149" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="150" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="151" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="152" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="153" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="154" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="155" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="156" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="157" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="158" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="159" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="160" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="161" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="162" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="163" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="164" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="165" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="166" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="167" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="168" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="169" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="170" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="171" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="172" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="173" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="174" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="175" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="176" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="177" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="178" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="179" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="180" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="181" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="182" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="183" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="184" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="185" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="186" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="187" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="188" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="189" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="190" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="191" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="192" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="193" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="194" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="195" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="196" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="197" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="198" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="199" spans="3:8" x14ac:dyDescent="0.25"/>
+    <row r="200" spans="3:8" x14ac:dyDescent="0.25"/>
   </sheetData>
   <dataValidations count="6">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="C10:C200">
@@ -2680,17 +2722,17 @@
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="C2:C200">
       <formula1>"Pulsador,Test,Verdad o mentira,Dos verdades y una mentira,Votación,Estimación,Parar el contador,Duelo de reflejos,Libre"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="F10:F200">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="F10:G200">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="F2:F200">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="F2:G200">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="G10:G200">
-      <formula1>"Noche de luna,Cementerio,Bosque encantado,Huerto de calabazas,Laboratorio,Mansión encantada,Telaraña,Aquelarre,Cripta helada,Tormenta"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="H10:H200">
+      <formula1>"Noche de luna,Cementerio,Bosque encantado,Huerto de calabazas,Laboratorio,Mansión encantada,Telaraña,Aquelarre,Cripta helada,Tormenta,Plató millonario"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="G2:G200">
-      <formula1>"Noche de luna,Cementerio,Bosque encantado,Huerto de calabazas,Laboratorio,Mansión encantada,Telaraña,Aquelarre,Cripta helada,Tormenta"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="H2:H200">
+      <formula1>"Noche de luna,Cementerio,Bosque encantado,Huerto de calabazas,Laboratorio,Mansión encantada,Telaraña,Aquelarre,Cripta helada,Tormenta,Plató millonario"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2713,26 +2755,26 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.25"/>
@@ -2961,23 +3003,23 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -2985,7 +3027,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -2993,7 +3035,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -3001,7 +3043,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -3009,7 +3051,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -3017,15 +3059,15 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B8" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B9">
         <v>20</v>
@@ -3054,64 +3096,64 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C4" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25"/>
@@ -3336,71 +3378,68 @@
   <sheetPr>
     <tabColor rgb="FF2E7D32"/>
   </sheetPr>
-  <dimension ref="A1:I200"/>
+  <dimension ref="A1:H200"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
     <col min="3" max="6" width="22" customWidth="1"/>
-    <col min="7" max="8" width="10" customWidth="1"/>
-    <col min="9" max="9" width="40" customWidth="1"/>
+    <col min="7" max="7" width="10" customWidth="1"/>
+    <col min="8" max="8" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F1" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E2" t="s">
+        <v>89</v>
+      </c>
+      <c r="F2" t="s">
+        <v>76</v>
+      </c>
+      <c r="G2" t="s">
         <v>81</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" t="s">
-        <v>85</v>
-      </c>
-      <c r="C2" t="s">
-        <v>86</v>
-      </c>
-      <c r="D2" t="s">
-        <v>87</v>
-      </c>
-      <c r="E2" t="s">
-        <v>88</v>
-      </c>
-      <c r="F2" t="s">
-        <v>89</v>
-      </c>
-      <c r="G2" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B3" t="s">
         <v>90</v>
@@ -3414,15 +3453,59 @@
       <c r="E3" t="s">
         <v>93</v>
       </c>
+      <c r="F3" t="s">
+        <v>94</v>
+      </c>
       <c r="G3" t="s">
-        <v>80</v>
-      </c>
-      <c r="H3">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25"/>
+        <v>81</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D4" t="s">
+        <v>97</v>
+      </c>
+      <c r="E4" t="s">
+        <v>98</v>
+      </c>
+      <c r="F4" t="s">
+        <v>99</v>
+      </c>
+      <c r="G4" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" t="s">
+        <v>100</v>
+      </c>
+      <c r="C5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D5" t="s">
+        <v>102</v>
+      </c>
+      <c r="E5" t="s">
+        <v>103</v>
+      </c>
+      <c r="F5" t="s">
+        <v>104</v>
+      </c>
+      <c r="G5" t="s">
+        <v>82</v>
+      </c>
+    </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25"/>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25"/>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25"/>
@@ -3654,35 +3737,35 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B2" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
       <c r="C2" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B3" t="s">
-        <v>97</v>
+        <v>108</v>
       </c>
       <c r="C3" t="s">
-        <v>98</v>
+        <v>109</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25"/>
@@ -3918,39 +4001,39 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>100</v>
+        <v>111</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>101</v>
+        <v>112</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>98</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B2" t="s">
-        <v>103</v>
+        <v>114</v>
       </c>
       <c r="C2" t="s">
-        <v>104</v>
+        <v>115</v>
       </c>
       <c r="D2" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
       <c r="E2" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="F2">
         <v>2</v>
@@ -4189,26 +4272,26 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>107</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B3" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Presentación del concurso y de equipos, millonario por dificultad y conexión más robusta
- Antes de empezar: preparación (archivos y mando) → título con su canción →
  conexión de jugadores → «Equipo A contra equipo B» con su música.
- Millonario: 2 fáciles, 2 medias y 2 difíciles (columna «Dificultad»), que
  valen 1 · 3 · 5; cada una con la música de su dificultad.
- Conexión: los TURN gratuitos de PeerJS ya no existen; el móvil y la tele
  explican por qué no conecta. Tras estar en segundo plano (o dos fallos
  seguidos) se rehace la conexión entera; el mando no se rinde si no encuentra
  la sala. La petición de mando ya no queda detrás del título.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantilla-concurso.xlsx
+++ b/public/plantilla-concurso.xlsx
@@ -227,6 +227,13 @@
     <comment ref="H1" authorId="0">
       <text>
         <r>
+          <t>Su música y sus puntos (columna Puntos de la pestaña Concurso: fácil, media, difícil, p. ej. 1,3,5). Vacía = por tercios.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0">
+      <text>
+        <r>
           <t>Opcional: dirección web de una imagen.</t>
         </r>
       </text>
@@ -277,7 +284,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="162">
   <si>
     <t>CÓMO RELLENAR ESTA PLANTILLA</t>
   </si>
@@ -366,6 +373,9 @@
     <t>¿Quién quiere ser millonario? Uno cada vez; vuestro portavoz decide el orden.</t>
   </si>
   <si>
+    <t>1,3,5</t>
+  </si>
+  <si>
     <t>¿Verdad o mentira?</t>
   </si>
   <si>
@@ -534,6 +544,9 @@
     <t>Correcta</t>
   </si>
   <si>
+    <t>Dificultad</t>
+  </si>
+  <si>
     <t>Imagen</t>
   </si>
   <si>
@@ -549,6 +562,24 @@
     <t>Siete</t>
   </si>
   <si>
+    <t>Fácil</t>
+  </si>
+  <si>
+    <t>¿De qué color es el caballo blanco de Santiago?</t>
+  </si>
+  <si>
+    <t>Negro</t>
+  </si>
+  <si>
+    <t>Marrón</t>
+  </si>
+  <si>
+    <t>Blanco</t>
+  </si>
+  <si>
+    <t>Gris</t>
+  </si>
+  <si>
     <t>¿En qué año llegó el hombre a la Luna?</t>
   </si>
   <si>
@@ -564,6 +595,24 @@
     <t>1975</t>
   </si>
   <si>
+    <t>Media</t>
+  </si>
+  <si>
+    <t>¿Cuál es el planeta más grande?</t>
+  </si>
+  <si>
+    <t>Saturno</t>
+  </si>
+  <si>
+    <t>Neptuno</t>
+  </si>
+  <si>
+    <t>Júpiter</t>
+  </si>
+  <si>
+    <t>Urano</t>
+  </si>
+  <si>
     <t>¿Cuál es la capital de provincia española que está a más altura?</t>
   </si>
   <si>
@@ -579,19 +628,22 @@
     <t>Ávila</t>
   </si>
   <si>
-    <t>¿Cuál es el planeta más grande?</t>
-  </si>
-  <si>
-    <t>Saturno</t>
-  </si>
-  <si>
-    <t>Neptuno</t>
-  </si>
-  <si>
-    <t>Júpiter</t>
-  </si>
-  <si>
-    <t>Urano</t>
+    <t>Difícil</t>
+  </si>
+  <si>
+    <t>¿Qué elemento químico tiene el símbolo W?</t>
+  </si>
+  <si>
+    <t>Wolframio</t>
+  </si>
+  <si>
+    <t>Vanadio</t>
+  </si>
+  <si>
+    <t>Osmio</t>
+  </si>
+  <si>
+    <t>Wiconio</t>
   </si>
   <si>
     <t>Afirmación</t>
@@ -1225,50 +1277,50 @@
         <v>15</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>120</v>
+        <v>135</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>121</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B2" t="s">
-        <v>122</v>
+        <v>137</v>
       </c>
       <c r="C2">
         <v>910</v>
       </c>
       <c r="D2" t="s">
-        <v>123</v>
+        <v>138</v>
       </c>
       <c r="E2" t="s">
-        <v>124</v>
+        <v>139</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B3" t="s">
-        <v>125</v>
+        <v>140</v>
       </c>
       <c r="C3">
         <v>120</v>
       </c>
       <c r="D3" t="s">
-        <v>126</v>
+        <v>141</v>
       </c>
       <c r="E3" t="s">
-        <v>127</v>
+        <v>142</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25"/>
@@ -1507,35 +1559,35 @@
         <v>15</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>128</v>
+        <v>143</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>129</v>
+        <v>144</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>130</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B2">
         <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>131</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B3">
         <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>132</v>
+        <v>147</v>
       </c>
       <c r="D3">
         <v>3</v>
@@ -1543,13 +1595,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B4">
         <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>133</v>
+        <v>148</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25"/>
@@ -1787,21 +1839,21 @@
         <v>15</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>134</v>
+        <v>149</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>135</v>
+        <v>150</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B2">
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>136</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25"/>
@@ -2043,16 +2095,16 @@
         <v>15</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>137</v>
+        <v>152</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>138</v>
+        <v>153</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>135</v>
+        <v>150</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>18</v>
@@ -2060,36 +2112,36 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B2" t="s">
-        <v>139</v>
+        <v>154</v>
       </c>
       <c r="C2" t="s">
-        <v>140</v>
+        <v>155</v>
       </c>
       <c r="D2" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
       <c r="E2" t="s">
-        <v>142</v>
+        <v>157</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
-        <v>143</v>
+        <v>158</v>
       </c>
       <c r="C3" t="s">
-        <v>144</v>
+        <v>159</v>
       </c>
       <c r="D3" t="s">
-        <v>145</v>
+        <v>160</v>
       </c>
       <c r="E3" t="s">
-        <v>146</v>
+        <v>161</v>
       </c>
       <c r="F3">
         <v>5</v>
@@ -2395,8 +2447,8 @@
       <c r="D3" t="s">
         <v>28</v>
       </c>
-      <c r="E3">
-        <v>2</v>
+      <c r="E3" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -2404,13 +2456,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2421,13 +2473,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2438,16 +2490,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -2455,16 +2507,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" t="s">
         <v>39</v>
-      </c>
-      <c r="C7" t="s">
-        <v>40</v>
-      </c>
-      <c r="D7" t="s">
-        <v>41</v>
-      </c>
-      <c r="E7" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -2472,16 +2524,16 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -2489,13 +2541,13 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2506,22 +2558,22 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C10" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E10">
         <v>3</v>
       </c>
       <c r="F10" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11" spans="3:8" x14ac:dyDescent="0.25"/>
@@ -2755,26 +2807,26 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.25"/>
@@ -3003,23 +3055,23 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -3027,7 +3079,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -3035,7 +3087,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -3043,7 +3095,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -3051,7 +3103,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -3059,15 +3111,15 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B9">
         <v>20</v>
@@ -3099,16 +3151,16 @@
         <v>15</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -3116,13 +3168,13 @@
         <v>22</v>
       </c>
       <c r="B2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -3130,13 +3182,13 @@
         <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -3144,16 +3196,16 @@
         <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25"/>
@@ -3378,331 +3430,397 @@
   <sheetPr>
     <tabColor rgb="FF2E7D32"/>
   </sheetPr>
-  <dimension ref="A1:H200"/>
+  <dimension ref="A1:I200"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
     <col min="3" max="6" width="22" customWidth="1"/>
     <col min="7" max="7" width="10" customWidth="1"/>
-    <col min="8" max="8" width="40" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="9" max="9" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>26</v>
       </c>
       <c r="B2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G2" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+      <c r="H2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E3" t="s">
+        <v>96</v>
+      </c>
+      <c r="F3" t="s">
+        <v>97</v>
+      </c>
+      <c r="G3" t="s">
+        <v>83</v>
+      </c>
+      <c r="H3" t="s">
         <v>92</v>
       </c>
-      <c r="E3" t="s">
-        <v>93</v>
-      </c>
-      <c r="F3" t="s">
-        <v>94</v>
-      </c>
-      <c r="G3" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>26</v>
       </c>
       <c r="B4" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C4" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="D4" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="E4" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="F4" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="G4" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+      <c r="H4" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>26</v>
       </c>
       <c r="B5" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C5" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="D5" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="E5" t="s">
+        <v>107</v>
+      </c>
+      <c r="F5" t="s">
+        <v>108</v>
+      </c>
+      <c r="G5" t="s">
+        <v>83</v>
+      </c>
+      <c r="H5" t="s">
         <v>103</v>
       </c>
-      <c r="F5" t="s">
-        <v>104</v>
-      </c>
-      <c r="G5" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="153" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="156" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="157" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="158" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="159" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="160" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="161" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="162" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="163" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="164" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="165" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="166" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="167" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="168" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="169" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="170" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="171" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="172" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="173" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="174" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="175" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="176" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="177" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="178" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="179" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="180" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="181" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="182" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="183" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="184" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="185" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="186" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="187" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="188" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="189" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="190" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="191" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="192" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="193" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="194" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="195" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="196" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="197" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="198" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="199" spans="1:7" x14ac:dyDescent="0.25"/>
-    <row r="200" spans="1:7" x14ac:dyDescent="0.25"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" t="s">
+        <v>109</v>
+      </c>
+      <c r="C6" t="s">
+        <v>110</v>
+      </c>
+      <c r="D6" t="s">
+        <v>111</v>
+      </c>
+      <c r="E6" t="s">
+        <v>112</v>
+      </c>
+      <c r="F6" t="s">
+        <v>113</v>
+      </c>
+      <c r="G6" t="s">
+        <v>84</v>
+      </c>
+      <c r="H6" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" t="s">
+        <v>115</v>
+      </c>
+      <c r="C7" t="s">
+        <v>116</v>
+      </c>
+      <c r="D7" t="s">
+        <v>117</v>
+      </c>
+      <c r="E7" t="s">
+        <v>118</v>
+      </c>
+      <c r="F7" t="s">
+        <v>119</v>
+      </c>
+      <c r="G7" t="s">
+        <v>81</v>
+      </c>
+      <c r="H7" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="112" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="113" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="114" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="115" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="116" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="117" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="118" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="119" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="120" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="121" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="122" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="123" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="124" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="125" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="126" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="127" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="128" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="129" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="130" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="131" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="132" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="133" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="134" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="135" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="136" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="137" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="138" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="139" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="140" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="141" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="142" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="143" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="144" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="145" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="146" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="147" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="148" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="149" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="150" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="151" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="152" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="153" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="154" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="155" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="156" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="157" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="158" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="159" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="160" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="161" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="162" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="163" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="164" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="165" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="166" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="167" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="168" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="169" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="170" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="171" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="172" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="173" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="174" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="175" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="176" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="177" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="178" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="179" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="180" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="181" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="182" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="183" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="184" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="185" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="186" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="187" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="188" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="189" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="190" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="191" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="192" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="193" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="194" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="195" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="196" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="197" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="198" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="199" spans="1:8" x14ac:dyDescent="0.25"/>
+    <row r="200" spans="1:8" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <dataValidations count="4">
+  <dataValidations count="6">
     <dataValidation type="list" allowBlank="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="A10:A200">
       <formula1>Concurso!$B$2:$B$100</formula1>
     </dataValidation>
@@ -3714,6 +3832,12 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="G2:G200">
       <formula1>"A,B,C,D"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="H10:H200">
+      <formula1>"Fácil,Media,Difícil"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="H2:H200">
+      <formula1>"Fácil,Media,Difícil"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3740,32 +3864,32 @@
         <v>15</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B2" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="C2" t="s">
-        <v>107</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B3" t="s">
-        <v>108</v>
+        <v>123</v>
       </c>
       <c r="C3" t="s">
-        <v>109</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25"/>
@@ -4004,36 +4128,36 @@
         <v>15</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>109</v>
+        <v>124</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B2" t="s">
-        <v>114</v>
+        <v>129</v>
       </c>
       <c r="C2" t="s">
-        <v>115</v>
+        <v>130</v>
       </c>
       <c r="D2" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="E2" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="F2">
         <v>2</v>
@@ -4275,23 +4399,23 @@
         <v>15</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>118</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B3" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25"/>

</xml_diff>